<commit_message>
Address code review comments: helper fn, error handling, clarifying comments, docs fix
Agent-Logs-Url: https://github.com/peetee09/Dashboard-DMS-v0.0.1-beta/sessions/f1d70600-15de-42d3-b20f-3d758395bc80

Co-authored-by: peetee09 <93839860+peetee09@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KPI_Workbook.xlsx
+++ b/KPI_Workbook.xlsx
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="8" t="n">
-        <v>46137.3094985277</v>
+        <v>46137.31100720354</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         <v>10</v>
       </c>
       <c r="I2" s="8" t="n">
-        <v>46137.30949851077</v>
+        <v>46137.31100718575</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
chore: start audit and improvements
Agent-Logs-Url: https://github.com/peetee09/Dashboard-DMS-v0.0.1-beta/sessions/c39e0d83-2e49-4e19-8667-0ebccf842a2a

Co-authored-by: peetee09 <93839860+peetee09@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KPI_Workbook.xlsx
+++ b/KPI_Workbook.xlsx
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="8" t="n">
-        <v>46137.31100720354</v>
+        <v>46137.32097220042</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         <v>10</v>
       </c>
       <c r="I2" s="8" t="n">
-        <v>46137.31100718575</v>
+        <v>46137.32097217493</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
fix: address code review feedback - comments, formula clarity, dynamic button positioning
Agent-Logs-Url: https://github.com/peetee09/Dashboard-DMS-v0.0.1-beta/sessions/c39e0d83-2e49-4e19-8667-0ebccf842a2a

Co-authored-by: peetee09 <93839860+peetee09@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/KPI_Workbook.xlsx
+++ b/KPI_Workbook.xlsx
@@ -2979,7 +2979,7 @@
         <v>10</v>
       </c>
       <c r="I2" s="62" t="n">
-        <v>46137.32682931781</v>
+        <v>46137.33146576225</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
@@ -3152,7 +3152,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="62" t="n">
-        <v>46137.32682934483</v>
+        <v>46137.33146578698</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>

</xml_diff>